<commit_message>
fix: finalize month-year analysis and submission deliverables
</commit_message>
<xml_diff>
--- a/PROJECT/BISM2202_OUTPUT/COMMON/analysis_results.xlsx
+++ b/PROJECT/BISM2202_OUTPUT/COMMON/analysis_results.xlsx
@@ -40,7 +40,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Q06'!$A$1:$H$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Q07'!$A$1:$H$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Q08'!$A$1:$H$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Q09'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Q09'!$A$1:$H$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Q10'!$A$1:$H$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Q11'!$A$1:$H$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Q12'!$A$1:$H$9</definedName>
@@ -951,7 +951,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Order volume trend across Order Month</t>
+          <t>Order volume trend by Month-Year</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Order Month</t>
+          <t>Month-Year</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Month Number ascending</t>
+          <t>Month-Year ascending</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -986,11 +986,11 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Aggregated across all years per wording; source covers 2024-01 to 2026-07.</t>
+          <t>One point per calendar month; 31 months from 2024-01 through 2026-07.</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11">
@@ -1535,15 +1535,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1593,7 +1593,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Order volume trend across Order Month</t>
+          <t>Order volume trend by Month-Year</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Order Month</t>
+          <t>Month-Year</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Month Number ascending</t>
+          <t>Month-Year ascending</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Aggregated across all years per wording; source covers 2024-01 to 2026-07.</t>
+          <t>One point per calendar month; 31 months from 2024-01 through 2026-07.</t>
         </is>
       </c>
     </row>
@@ -1645,12 +1645,12 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Month Number</t>
+          <t>Month-Year</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Order Month</t>
+          <t>Month-Year Start</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1665,16 +1665,18 @@
       <c r="H4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>1</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>January</t>
+          <t>2024-01-01T00:00:00</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>88</v>
+        <v>26</v>
       </c>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
@@ -1683,16 +1685,18 @@
       <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>2</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>February</t>
+          <t>2024-02-01T00:00:00</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
@@ -1701,16 +1705,18 @@
       <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>3</v>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>March</t>
+          <t>2024-03-01T00:00:00</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>94</v>
+        <v>32</v>
       </c>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
@@ -1719,16 +1725,18 @@
       <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>4</v>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>April</t>
+          <t>2024-04-01T00:00:00</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>91</v>
+        <v>31</v>
       </c>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
@@ -1737,16 +1745,18 @@
       <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>5</v>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>2024-05-01T00:00:00</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
@@ -1755,16 +1765,18 @@
       <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>6</v>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>June</t>
+          <t>2024-06-01T00:00:00</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>91</v>
+        <v>11</v>
       </c>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
@@ -1773,16 +1785,18 @@
       <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>7</v>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>July</t>
+          <t>2024-07-01T00:00:00</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
@@ -1791,16 +1805,18 @@
       <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>8</v>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>August</t>
+          <t>2024-08-01T00:00:00</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>117</v>
+        <v>86</v>
       </c>
       <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="n"/>
@@ -1809,16 +1825,18 @@
       <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>9</v>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>September</t>
+          <t>2024-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="n"/>
@@ -1827,16 +1845,18 @@
       <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>10</v>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>October</t>
+          <t>2024-10-01T00:00:00</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
@@ -1845,16 +1865,18 @@
       <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>11</v>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>November</t>
+          <t>2024-11-01T00:00:00</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
@@ -1863,16 +1885,18 @@
       <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>12</v>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>December</t>
+          <t>2024-12-01T00:00:00</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
@@ -1880,8 +1904,388 @@
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2025-01-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2025-02-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2025-03-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2025-04-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2025-06-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2025-07-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2025-08-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2025-09-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2025-10-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01T00:00:00</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:H35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: finalize corrected BISM2202 A and B submissions
</commit_message>
<xml_diff>
--- a/PROJECT/BISM2202_OUTPUT/COMMON/analysis_results.xlsx
+++ b/PROJECT/BISM2202_OUTPUT/COMMON/analysis_results.xlsx
@@ -510,7 +510,7 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="29" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
@@ -951,7 +951,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Order volume trend by Month-Year</t>
+          <t>How does order volume trend across Order Month?</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Month-Year</t>
+          <t>Order Month Start</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Month-Year ascending</t>
+          <t>Order Month Start ascending</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1486,12 +1486,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Reuses Q01/Q12/Q14/Q16/Q17/Q19 metrics</t>
+          <t>Reuses Q13/Q14/Q16 metrics</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Restaurant; Traffic; Hour; Location; Pizza Type; Payment</t>
+          <t>Restaurant; Traffic Level; Order Hour</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1538,12 +1538,12 @@
   <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1593,7 +1593,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Order volume trend by Month-Year</t>
+          <t>How does order volume trend across Order Month?</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Month-Year</t>
+          <t>Order Month Start</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Month-Year ascending</t>
+          <t>Order Month Start ascending</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -5541,8 +5541,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -5600,12 +5600,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Reuses Q01/Q12/Q14/Q16/Q17/Q19 metrics</t>
+          <t>Reuses Q13/Q14/Q16 metrics</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Restaurant; Traffic; Hour; Location; Pizza Type; Payment</t>
+          <t>Restaurant; Traffic Level; Order Hour</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">

</xml_diff>